<commit_message>
📄 Update to Record_Sept-22-2.xlsx (2382/9888 09-08 entry masked → 42 open pairs)
</commit_message>
<xml_diff>
--- a/data/Record_Sept-22.xlsx
+++ b/data/Record_Sept-22.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="20">
   <si>
     <t>Base</t>
   </si>
@@ -3576,11 +3576,11 @@
       </c>
     </row>
     <row r="178" ht="15.75" customHeight="1">
-      <c r="A178" s="13">
-        <v>80.8</v>
-      </c>
-      <c r="B178" s="4">
-        <v>104.8</v>
+      <c r="A178" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B178" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="H178" s="5" t="str">
         <f>H176-H177</f>

</xml_diff>